<commit_message>
Improved Informazioni.xlsl, improved CIS description
</commit_message>
<xml_diff>
--- a/docs/assignment/informazioni.xlsx
+++ b/docs/assignment/informazioni.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\IGES\Progetto\docs\assignment\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\Desktop\Luciano\IGES\smartbugs\docs\assignment\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBE0ECD-4A5B-452D-A8A6-E520E5A7DEB3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13070F1-6373-411A-9085-4F43AA07E6CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="progetto" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
   <si>
     <t>Matricola</t>
   </si>
@@ -63,9 +63,6 @@
     <t>Email unisa</t>
   </si>
   <si>
-    <t>Noma Progetto</t>
-  </si>
-  <si>
     <t>0522501684</t>
   </si>
   <si>
@@ -79,6 +76,15 @@
   </si>
   <si>
     <t>SmartBugs</t>
+  </si>
+  <si>
+    <t>https://github.com/Luciano-Bercini-Unisa/IGES-Project</t>
+  </si>
+  <si>
+    <t>SmartBugs Intelligent Tool Selection</t>
+  </si>
+  <si>
+    <t>Estensione del framework SmartBugs con un meccanismo di selezione automatica dei tool di analisi basato su feature extraction e modelli di machine learning.</t>
   </si>
 </sst>
 </file>
@@ -150,7 +156,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="36">
+  <cellStyleXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -187,16 +193,18 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="36"/>
   </cellXfs>
-  <cellStyles count="36">
+  <cellStyles count="37">
     <cellStyle name="Followed Hyperlink" xfId="2" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="4" builtinId="9" hidden="1"/>
     <cellStyle name="Followed Hyperlink" xfId="6" builtinId="9" hidden="1"/>
@@ -232,6 +240,7 @@
     <cellStyle name="Hyperlink" xfId="3" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="5" builtinId="8" hidden="1"/>
     <cellStyle name="Hyperlink" xfId="7" builtinId="8" hidden="1"/>
+    <cellStyle name="Hyperlink" xfId="36" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -569,10 +578,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.625" customWidth="1"/>
+    <col min="1" max="1" width="32.625" customWidth="1"/>
     <col min="2" max="2" width="47.625" customWidth="1"/>
     <col min="3" max="3" width="36" customWidth="1"/>
   </cols>
@@ -588,7 +597,21 @@
         <v>5</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>14</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{127D4EC5-D3F1-4FED-8EB3-47E633AA9716}"/>
+  </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -617,24 +640,24 @@
         <v>6</v>
       </c>
       <c r="E1" s="5" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>